<commit_message>
Mise à jour des résultats du script
</commit_message>
<xml_diff>
--- a/result/Data.xlsx
+++ b/result/Data.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D492"/>
+  <dimension ref="A1:D493"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8942,6 +8942,26 @@
         <v>4</v>
       </c>
     </row>
+    <row r="493">
+      <c r="A493" t="inlineStr">
+        <is>
+          <t>2026-03-03</t>
+        </is>
+      </c>
+      <c r="B493" t="inlineStr">
+        <is>
+          <t>Rien ne nous concerne aujourd'hui !</t>
+        </is>
+      </c>
+      <c r="C493" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="D493" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>